<commit_message>
Add start date and end date for layer 4
</commit_message>
<xml_diff>
--- a/src/WBS_import_template.xlsx
+++ b/src/WBS_import_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="52">
   <si>
     <t>Layer</t>
   </si>
@@ -122,7 +122,7 @@
     <t>Name, Phase, Deliverable, Epic</t>
   </si>
   <si>
-    <t>Start Sprint, End Sprint, Status, ID</t>
+    <t>Start Date, End Date, Start Sprint, End Sprint, Status, ID</t>
   </si>
   <si>
     <t>Dates</t>
@@ -144,6 +144,12 @@
   </si>
   <si>
     <t>Blank sprint fields mean unscheduled. If supplied, each sprint range must fit its immediate parent range.</t>
+  </si>
+  <si>
+    <t>Task dates</t>
+  </si>
+  <si>
+    <t>Optional paired working-day dates inside the epic and phase. Dates derive sprint numbers. When both are supplied they must agree. Sprint-only tasks keep their full sprint range.</t>
   </si>
   <si>
     <t>Sprint numbers</t>
@@ -756,7 +762,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -896,6 +902,17 @@
         <v>14</v>
       </c>
     </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B13" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>